<commit_message>
Updated MPCbS using PNE report
</commit_message>
<xml_diff>
--- a/InputData/elec/MPCbS/Max Potential Capacity by Source.xlsx
+++ b/InputData/elec/MPCbS/Max Potential Capacity by Source.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10727"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-brazil-cpl/InputData/elec/MPCbS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saido\Documents\eps-brazil-cpl\InputData\elec\MPCbS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3287EE27-3CDF-6046-A158-DF9E360CD9AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="765" windowWidth="34200" windowHeight="21375" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Data" sheetId="2" r:id="rId2"/>
     <sheet name="MPCbS" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="43">
   <si>
     <t>Source:</t>
   </si>
@@ -131,13 +130,46 @@
   </si>
   <si>
     <t>EPE - Empresa de Pesquisa Energética</t>
+  </si>
+  <si>
+    <t>PNE report</t>
+  </si>
+  <si>
+    <t>Offshore wind</t>
+  </si>
+  <si>
+    <t>Lignite</t>
+  </si>
+  <si>
+    <t>Solar thermal</t>
+  </si>
+  <si>
+    <t>Solar PV</t>
+  </si>
+  <si>
+    <t>Onshore wind</t>
+  </si>
+  <si>
+    <t>Hydro</t>
+  </si>
+  <si>
+    <t>Nuclear</t>
+  </si>
+  <si>
+    <t>Basis</t>
+  </si>
+  <si>
+    <t>Potential capacity (MW)</t>
+  </si>
+  <si>
+    <t>Power plant type</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,8 +193,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -181,8 +226,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor rgb="FF003366"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -190,12 +241,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -208,9 +274,17 @@
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -227,9 +301,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -267,9 +341,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -304,7 +378,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -339,7 +413,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -512,19 +586,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -532,49 +606,49 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
         <v>2018</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>25</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" xr:uid="{ECCBFAB6-316C-4985-BA85-6CA058C03D6E}"/>
+    <hyperlink ref="B6" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
@@ -582,18 +656,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A2:D22"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.6640625" customWidth="1"/>
-    <col min="2" max="3" width="24.6640625" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" customWidth="1"/>
+    <col min="2" max="3" width="24.7109375" customWidth="1"/>
     <col min="5" max="5" width="71" customWidth="1"/>
-    <col min="6" max="6" width="16.33203125" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -605,7 +679,7 @@
       </c>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -616,7 +690,7 @@
         <v>1760000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -628,7 +702,7 @@
       </c>
       <c r="D4" s="4"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -639,7 +713,7 @@
         <v>5140000</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -650,7 +724,7 @@
         <v>3400000</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -661,7 +735,7 @@
         <v>1400000</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -672,7 +746,7 @@
         <v>2000000</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -683,7 +757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -694,7 +768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>28</v>
       </c>
@@ -702,12 +776,100 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>29</v>
       </c>
       <c r="B13" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="11">
+        <v>12395</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="11">
+        <v>176000</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="11">
+        <v>440500</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="11">
+        <v>307000</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="11">
+        <v>203306</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="11">
+        <v>27397</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="11">
+        <v>57000</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -716,18 +878,18 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="27.33203125" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -735,7 +897,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -744,7 +906,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -753,7 +915,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -762,43 +924,43 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="7">
-        <f>Data!C3</f>
-        <v>1760000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+        <f>Data!B17</f>
+        <v>176000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="7">
-        <f>Data!C4</f>
-        <v>1790000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+        <f>Data!B18</f>
+        <v>440500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="7">
-        <f>Data!C6</f>
-        <v>3400000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+        <f>Data!B19</f>
+        <v>307000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="7">
-        <f>Data!C7</f>
-        <v>1400000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+        <f>Data!B20</f>
+        <v>203306</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -807,7 +969,7 @@
         <v>2000000</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -816,7 +978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -825,7 +987,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -834,7 +996,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -843,16 +1005,16 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="7">
-        <f>Data!C5</f>
-        <v>5140000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+        <f>Data!B22</f>
+        <v>57000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -861,7 +1023,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -870,7 +1032,7 @@
         <v>9000000000000</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>

</xml_diff>